<commit_message>
Criado metodo abrirNavegador na classe Page
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>EXECUTE</t>
   </si>
@@ -106,9 +106,6 @@
   </si>
   <si>
     <t>Delhi</t>
-  </si>
-  <si>
-    <t>Não</t>
   </si>
   <si>
     <t>Lisa</t>
@@ -826,7 +823,7 @@
       <c r="I2" s="2">
         <v>23</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K2" s="2">
@@ -841,7 +838,7 @@
       <c r="N2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" s="2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="2" t="s">
@@ -852,8 +849,8 @@
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="2" t="s">
-        <v>30</v>
+      <c r="A3" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="B3" s="2">
         <v>2</v>
@@ -862,16 +859,16 @@
         <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="H3" s="2">
         <v>16991524631</v>
@@ -879,34 +876,34 @@
       <c r="I3" s="2">
         <v>9</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>34</v>
+      <c r="J3" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="K3" s="2">
         <v>1984</v>
       </c>
       <c r="L3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="P3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="2" t="s">
-        <v>30</v>
+      <c r="A4" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="B4" s="2">
         <v>3</v>
@@ -915,16 +912,16 @@
         <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H4" s="2">
         <v>15984828279</v>
@@ -932,29 +929,29 @@
       <c r="I4" s="2">
         <v>19</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>43</v>
+      <c r="J4" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="K4" s="2">
         <v>1990</v>
       </c>
       <c r="L4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="P4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="Q4" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Concluido criação do cenario CT01
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -87,7 +87,7 @@
     <t>Male</t>
   </si>
   <si>
-    <t>Febuary</t>
+    <t>February</t>
   </si>
   <si>
     <t>Commerce</t>
@@ -228,10 +228,9 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -821,7 +820,7 @@
         <v>22</v>
       </c>
       <c r="H2" s="2">
-        <v>61973551338</v>
+        <v>6197355133</v>
       </c>
       <c r="I2" s="2">
         <v>23</v>
@@ -852,7 +851,7 @@
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B3" s="2">
@@ -874,7 +873,7 @@
         <v>33</v>
       </c>
       <c r="H3" s="2">
-        <v>16991524631</v>
+        <v>1699152463</v>
       </c>
       <c r="I3" s="2">
         <v>9</v>
@@ -905,7 +904,7 @@
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B4" s="2">
@@ -927,7 +926,7 @@
         <v>33</v>
       </c>
       <c r="H4" s="2">
-        <v>15984828279</v>
+        <v>1598482827</v>
       </c>
       <c r="I4" s="2">
         <v>19</v>

</xml_diff>

<commit_message>
Corrigido erro de report-html
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Cenários" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cenários" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -15,8 +15,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>EXECUTE</t>
   </si>
@@ -67,6 +89,12 @@
   </si>
   <si>
     <t>CITY</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>ERRO</t>
   </si>
   <si>
     <t>Sim</t>
@@ -172,36 +200,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11.000000"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.000000"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.499984740745262"/>
-        <bgColor theme="1" tint="0.499984740745262"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -209,30 +224,12 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -242,9 +239,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -536,7 +530,7 @@
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="New Office">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -544,39 +538,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface="Arial"/>
         <a:cs typeface="Arial"/>
       </a:majorFont>
@@ -595,371 +589,424 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr bwMode="auto"/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr bwMode="auto"/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col bestFit="1" min="1" max="1" width="8.421875"/>
-    <col bestFit="1" min="2" max="2" width="2.57421875"/>
-    <col bestFit="1" min="3" max="3" width="44.2109375"/>
-    <col bestFit="1" min="4" max="4" width="12.07421875"/>
-    <col bestFit="1" min="5" max="5" width="11.50390625"/>
-    <col bestFit="1" min="6" max="6" width="24.2109375"/>
-    <col bestFit="1" min="8" max="8" width="16.2109375"/>
-    <col min="9" max="10" width="16.2109375"/>
-    <col bestFit="1" min="11" max="11" width="15.2109375"/>
-    <col bestFit="1" min="12" max="12" width="9.921875"/>
-    <col bestFit="1" min="15" max="15" width="74.140625"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="14.25">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" ht="14.25">
-      <c r="A2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="2">
+    <row r="2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2">
+        <v>6197355133</v>
+      </c>
+      <c r="I2">
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2">
+        <v>1981</v>
+      </c>
+      <c r="L2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3">
+        <v>1699152463</v>
+      </c>
+      <c r="I3">
+        <v>11</v>
+      </c>
+      <c r="J3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3">
+        <v>1984</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="D4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="2">
-        <v>6197355133</v>
-      </c>
-      <c r="I2" s="2">
-        <v>23</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="2">
-        <v>1981</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" ht="14.25">
-      <c r="A3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="2">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1699152463</v>
-      </c>
-      <c r="I3" s="2">
-        <v>9</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K3" s="2">
-        <v>1984</v>
-      </c>
-      <c r="L3" s="2" t="s">
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" t="s">
         <v>35</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" ht="14.25">
-      <c r="A4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="2">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" s="2">
+      <c r="H4">
         <v>1598482827</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4">
         <v>19</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="K4" s="2">
+      <c r="J4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K4">
         <v>1990</v>
       </c>
-      <c r="L4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="N4" s="2" t="s">
+      <c r="L4" t="s">
         <v>46</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="M4" t="s">
         <v>47</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="N4" t="s">
         <v>48</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="O4" t="s">
         <v>49</v>
+      </c>
+      <c r="P4" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000014" footer="0.31496062000000014"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>

</xml_diff>